<commit_message>
new card combination, card effect and something
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Downloads\UNR\CS 425\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1A1589-505A-4D30-8ABB-1FB094C27371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F202DD9D-090F-403C-B824-E1B9AEF352CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,15 +62,6 @@
     <t>None</t>
   </si>
   <si>
-    <t>has fast speed. The player can attack twice. Damage is low</t>
-  </si>
-  <si>
-    <t>has average speed. Damage is average. *unique ability: bullet can shoot through multiple enemies*</t>
-  </si>
-  <si>
-    <t>has slow speed. Damage is high. *unique ability: bullets have a chance to dismember enemies, causing them to do less damage to the player*</t>
-  </si>
-  <si>
     <t>Rarity (0 = Common, 1 = Rare, 2 =VeryRare, 3 = Epic)</t>
   </si>
   <si>
@@ -78,6 +69,15 @@
   </si>
   <si>
     <t>Weapons</t>
+  </si>
+  <si>
+    <t>Inflicts 1 enemy damage with a 90% hit rate and a multiplier of 1.</t>
+  </si>
+  <si>
+    <t>Inflicts 1 enemy damage with a 100% hit rate and a multiplier of 1.1.</t>
+  </si>
+  <si>
+    <t>Inflicts All enemies damage with a 70% hit rate and a multiplier of 0.7.</t>
   </si>
 </sst>
 </file>
@@ -412,10 +412,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -433,7 +433,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -442,7 +442,7 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -454,7 +454,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -463,7 +463,7 @@
         <v>7</v>
       </c>
       <c r="F3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -475,7 +475,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -484,7 +484,7 @@
         <v>7</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
weaponValue update, excelReader weapon part updata
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Downloads\UNR\CS 425\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025fall\CS 425\Project\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F202DD9D-090F-403C-B824-E1B9AEF352CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409D8B11-B68A-4CB8-AEA8-A0797311C921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>ID</t>
   </si>
@@ -78,6 +78,24 @@
   </si>
   <si>
     <t>Inflicts All enemies damage with a 70% hit rate and a multiplier of 0.7.</t>
+  </si>
+  <si>
+    <t>WeaponLevel</t>
+  </si>
+  <si>
+    <t>MaxLevel</t>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>MaterialName</t>
+  </si>
+  <si>
+    <t>MaterialNeed</t>
+  </si>
+  <si>
+    <t>Whetstone</t>
   </si>
 </sst>
 </file>
@@ -395,16 +413,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
+    <col min="2" max="3" width="19.6328125" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" customWidth="1"/>
-    <col min="6" max="6" width="21.33203125" customWidth="1"/>
+    <col min="5" max="5" width="22.54296875" customWidth="1"/>
+    <col min="6" max="6" width="58.81640625" customWidth="1"/>
+    <col min="7" max="7" width="24.26953125" customWidth="1"/>
+    <col min="8" max="8" width="11.36328125" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" customWidth="1"/>
+    <col min="11" max="11" width="16.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -423,10 +445,25 @@
       <c r="F1" t="s">
         <v>3</v>
       </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2">
-        <f t="shared" ref="A2:A4" si="0">ROW()-2</f>
+        <f t="shared" ref="A2:A6" si="0">ROW()-2</f>
         <v>0</v>
       </c>
       <c r="B2" t="s">
@@ -444,14 +481,26 @@
       <c r="F2" t="s">
         <v>12</v>
       </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -463,16 +512,31 @@
         <v>7</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>15</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -484,7 +548,82 @@
         <v>7</v>
       </c>
       <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
         <v>13</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add whetstone drop as a bonus after win a battle
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025fall\CS 425\Project\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025fall\CS 425\Team_Project\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409D8B11-B68A-4CB8-AEA8-A0797311C921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E218B422-EE90-49BB-AF26-88C016B969EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="21">
   <si>
     <t>ID</t>
   </si>
@@ -96,18 +96,29 @@
   </si>
   <si>
     <t>Whetstone</t>
+  </si>
+  <si>
+    <t>Whetstone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -135,7 +146,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -413,20 +424,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="3" width="19.6328125" customWidth="1"/>
+    <col min="2" max="3" width="19.625" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="22.54296875" customWidth="1"/>
-    <col min="6" max="6" width="58.81640625" customWidth="1"/>
-    <col min="7" max="7" width="24.26953125" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" customWidth="1"/>
-    <col min="10" max="10" width="17.26953125" customWidth="1"/>
-    <col min="11" max="11" width="16.453125" customWidth="1"/>
+    <col min="5" max="5" width="22.5" customWidth="1"/>
+    <col min="6" max="6" width="58.875" customWidth="1"/>
+    <col min="7" max="7" width="24.25" customWidth="1"/>
+    <col min="8" max="8" width="11.375" customWidth="1"/>
+    <col min="10" max="10" width="17.25" customWidth="1"/>
+    <col min="11" max="11" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -461,9 +472,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
-        <f t="shared" ref="A2:A6" si="0">ROW()-2</f>
+        <f t="shared" ref="A2:A10" si="0">ROW()-2</f>
         <v>0</v>
       </c>
       <c r="B2" t="s">
@@ -494,7 +505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -530,7 +541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -560,13 +571,13 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K4">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -595,38 +606,189 @@
       <c r="I5">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>28</v>
+      </c>
+      <c r="J6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>36</v>
+      </c>
+      <c r="J7" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
         <v>13</v>
       </c>
-      <c r="G6">
+      <c r="G8">
         <v>1</v>
       </c>
-      <c r="H6">
-        <v>3</v>
-      </c>
-      <c r="I6">
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8">
         <v>15</v>
       </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="I9">
+        <v>20</v>
+      </c>
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+      <c r="I10">
+        <v>25</v>
+      </c>
+      <c r="J10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change the description information of the task reminder
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/WeaponsValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025fall\CS 425\Team_Project\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2C0DEA-18C3-4AB3-B584-5F3689EE1D98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{195CAE13-6E33-450F-833F-D2567344A5AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,9 +77,6 @@
     <t>Inflicts 1 enemy damage with a 100% hit rate and a multiplier of 1.1.</t>
   </si>
   <si>
-    <t>Inflicts All enemies damage with a 70% hit rate and a multiplier of 0.7.</t>
-  </si>
-  <si>
     <t>WeaponLevel</t>
   </si>
   <si>
@@ -99,6 +96,10 @@
   </si>
   <si>
     <t>Whetstone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Deal 5 consecutive hits to the enemy. The hit rate for the first hit is 70%, and it decreases by 10% for each subsequent hit.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -457,19 +458,19 @@
         <v>3</v>
       </c>
       <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
         <v>14</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>15</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>16</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
@@ -535,7 +536,7 @@
         <v>15</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K3">
         <v>5</v>
@@ -571,7 +572,7 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
         <v>10</v>
@@ -640,7 +641,7 @@
         <v>28</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -676,7 +677,7 @@
         <v>36</v>
       </c>
       <c r="J7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K7">
         <v>10</v>
@@ -700,7 +701,7 @@
         <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -733,7 +734,7 @@
         <v>7</v>
       </c>
       <c r="F9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G9">
         <v>2</v>
@@ -745,7 +746,7 @@
         <v>25</v>
       </c>
       <c r="J9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K9">
         <v>6</v>
@@ -769,7 +770,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -781,7 +782,7 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K10">
         <v>12</v>

</xml_diff>